<commit_message>
Actualizar nombre de promotor en horarios.xlsx
</commit_message>
<xml_diff>
--- a/horarios.xlsx
+++ b/horarios.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Dreame\Desktop\Claude\Dreame\Turnos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3162802A-DA98-4C0B-847F-9337D859093A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73193F81-0317-4C83-B386-A988D5714BD1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -65,9 +65,6 @@
     <t>KARIN ANDREA NAVIA LILLO</t>
   </si>
   <si>
-    <t>JAVIER ANTONIA VERDUGO JARA</t>
-  </si>
-  <si>
     <t>ROMINA MANSILLA</t>
   </si>
   <si>
@@ -96,6 +93,9 @@
   </si>
   <si>
     <t>Libre</t>
+  </si>
+  <si>
+    <t>LESLIE SCHAAD</t>
   </si>
 </sst>
 </file>
@@ -609,7 +609,7 @@
   <sheetData>
     <row r="1" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B1" s="15" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C1" s="15"/>
       <c r="D1" s="15"/>
@@ -708,16 +708,16 @@
         <v>3</v>
       </c>
       <c r="B4" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C4" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D4" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E4" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F4" s="12">
         <v>0.4375</v>
@@ -757,16 +757,16 @@
         <v>4</v>
       </c>
       <c r="B5" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C5" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D5" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E5" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F5" s="12">
         <v>0.4375</v>
@@ -806,16 +806,16 @@
         <v>5</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C6" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D6" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E6" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F6" s="12">
         <v>0.4375</v>
@@ -861,16 +861,16 @@
         <v>0.79166666666666663</v>
       </c>
       <c r="D7" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E7" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F7" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="G7" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="H7" s="12">
         <v>0.41666666666666669</v>
@@ -904,16 +904,16 @@
         <v>7</v>
       </c>
       <c r="B8" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C8" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D8" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E8" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F8" s="12">
         <v>0.4375</v>
@@ -953,16 +953,16 @@
         <v>8</v>
       </c>
       <c r="B9" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C9" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D9" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E9" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F9" s="12">
         <v>0.4375</v>
@@ -999,19 +999,19 @@
     </row>
     <row r="10" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A10" s="6" t="s">
-        <v>9</v>
+        <v>19</v>
       </c>
       <c r="B10" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C10" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D10" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E10" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F10" s="12">
         <v>0.4375</v>
@@ -1048,19 +1048,19 @@
     </row>
     <row r="11" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A11" s="6" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B11" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C11" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D11" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E11" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F11" s="12">
         <v>0.4375</v>
@@ -1097,7 +1097,7 @@
     </row>
     <row r="12" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A12" s="6" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B12" s="12">
         <v>0.4375</v>
@@ -1112,16 +1112,16 @@
         <v>0.79166666666666663</v>
       </c>
       <c r="F12" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="G12" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="H12" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="I12" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="J12" s="12">
         <v>0.41666666666666669</v>
@@ -1146,19 +1146,19 @@
     </row>
     <row r="13" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A13" s="6" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B13" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C13" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D13" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E13" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F13" s="12">
         <v>0.4375</v>
@@ -1193,7 +1193,7 @@
     </row>
     <row r="14" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A14" s="6" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B14" s="12">
         <v>0.4375</v>
@@ -1202,16 +1202,16 @@
         <v>0.79166666666666663</v>
       </c>
       <c r="D14" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E14" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F14" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="G14" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="H14" s="12">
         <v>0.4375</v>
@@ -1240,19 +1240,19 @@
     </row>
     <row r="15" spans="1:18" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A15" s="14" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B15" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C15" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D15" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E15" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F15" s="12">
         <v>0.4375</v>
@@ -1287,7 +1287,7 @@
     </row>
     <row r="18" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B18" s="15" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C18" s="15"/>
       <c r="D18" s="15"/>
@@ -1386,10 +1386,10 @@
         <v>3</v>
       </c>
       <c r="B21" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C21" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D21" s="12">
         <v>0.4375</v>
@@ -1422,10 +1422,10 @@
         <v>0.83333333333333337</v>
       </c>
       <c r="N21" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="O21" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="22" spans="1:15" x14ac:dyDescent="0.3">
@@ -1433,10 +1433,10 @@
         <v>4</v>
       </c>
       <c r="B22" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C22" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D22" s="12">
         <v>0.4375</v>
@@ -1469,10 +1469,10 @@
         <v>0.83333333333333337</v>
       </c>
       <c r="N22" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="O22" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="23" spans="1:15" x14ac:dyDescent="0.3">
@@ -1480,10 +1480,10 @@
         <v>5</v>
       </c>
       <c r="B23" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C23" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D23" s="12">
         <v>0.4375</v>
@@ -1516,10 +1516,10 @@
         <v>0.83333333333333337</v>
       </c>
       <c r="N23" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="O23" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="24" spans="1:15" x14ac:dyDescent="0.3">
@@ -1527,10 +1527,10 @@
         <v>6</v>
       </c>
       <c r="B24" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C24" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D24" s="12">
         <v>0.4375</v>
@@ -1563,10 +1563,10 @@
         <v>0.83333333333333337</v>
       </c>
       <c r="N24" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="O24" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="25" spans="1:15" x14ac:dyDescent="0.3">
@@ -1574,10 +1574,10 @@
         <v>7</v>
       </c>
       <c r="B25" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C25" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D25" s="12">
         <v>0.4375</v>
@@ -1610,10 +1610,10 @@
         <v>0.83333333333333337</v>
       </c>
       <c r="N25" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="O25" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="26" spans="1:15" x14ac:dyDescent="0.3">
@@ -1621,10 +1621,10 @@
         <v>8</v>
       </c>
       <c r="B26" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C26" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D26" s="12">
         <v>0.4375</v>
@@ -1657,21 +1657,21 @@
         <v>0.83333333333333337</v>
       </c>
       <c r="N26" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="O26" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="27" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A27" s="6" t="s">
-        <v>9</v>
+        <v>19</v>
       </c>
       <c r="B27" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C27" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D27" s="12">
         <v>0.4375</v>
@@ -1704,21 +1704,21 @@
         <v>0.83333333333333337</v>
       </c>
       <c r="N27" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="O27" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="28" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A28" s="6" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B28" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C28" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D28" s="12">
         <v>0.4375</v>
@@ -1751,21 +1751,21 @@
         <v>0.83333333333333337</v>
       </c>
       <c r="N28" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="O28" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="29" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A29" s="6" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B29" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C29" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D29" s="12">
         <v>0.4375</v>
@@ -1798,21 +1798,21 @@
         <v>0.83333333333333337</v>
       </c>
       <c r="N29" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="O29" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="30" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A30" s="6" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B30" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C30" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D30" s="12">
         <v>0.4375</v>
@@ -1845,21 +1845,21 @@
         <v>0.83333333333333337</v>
       </c>
       <c r="N30" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="O30" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="31" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A31" s="6" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B31" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C31" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D31" s="12">
         <v>0.4375</v>
@@ -1892,21 +1892,21 @@
         <v>0.83333333333333337</v>
       </c>
       <c r="N31" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="O31" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="32" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A32" s="14" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B32" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C32" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D32" s="12">
         <v>0.4375</v>
@@ -1939,15 +1939,15 @@
         <v>0.83333333333333337</v>
       </c>
       <c r="N32" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="O32" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="35" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B35" s="15" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C35" s="15"/>
       <c r="D35" s="15"/>
@@ -2052,10 +2052,10 @@
         <v>0.79166666666666663</v>
       </c>
       <c r="D38" s="9" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E38" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F38" s="12">
         <v>0.4375</v>
@@ -2082,10 +2082,10 @@
         <v>0.83333333333333337</v>
       </c>
       <c r="N38" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="O38" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="39" spans="1:15" x14ac:dyDescent="0.3">
@@ -2099,10 +2099,10 @@
         <v>0.79166666666666663</v>
       </c>
       <c r="D39" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E39" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F39" s="12">
         <v>0.4375</v>
@@ -2129,10 +2129,10 @@
         <v>0.83333333333333337</v>
       </c>
       <c r="N39" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="O39" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="40" spans="1:15" x14ac:dyDescent="0.3">
@@ -2146,10 +2146,10 @@
         <v>0.79166666666666663</v>
       </c>
       <c r="D40" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E40" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F40" s="12">
         <v>0.4375</v>
@@ -2176,10 +2176,10 @@
         <v>0.83333333333333337</v>
       </c>
       <c r="N40" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="O40" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="41" spans="1:15" x14ac:dyDescent="0.3">
@@ -2193,10 +2193,10 @@
         <v>0.79166666666666663</v>
       </c>
       <c r="D41" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E41" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F41" s="12">
         <v>0.4375</v>
@@ -2223,10 +2223,10 @@
         <v>0.83333333333333337</v>
       </c>
       <c r="N41" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="O41" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="42" spans="1:15" x14ac:dyDescent="0.3">
@@ -2240,10 +2240,10 @@
         <v>0.79166666666666663</v>
       </c>
       <c r="D42" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E42" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F42" s="12">
         <v>0.4375</v>
@@ -2270,10 +2270,10 @@
         <v>0.83333333333333337</v>
       </c>
       <c r="N42" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="O42" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="43" spans="1:15" x14ac:dyDescent="0.3">
@@ -2287,10 +2287,10 @@
         <v>0.79166666666666663</v>
       </c>
       <c r="D43" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E43" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F43" s="12">
         <v>0.4375</v>
@@ -2317,15 +2317,15 @@
         <v>0.83333333333333337</v>
       </c>
       <c r="N43" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="O43" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="44" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A44" s="6" t="s">
-        <v>9</v>
+        <v>19</v>
       </c>
       <c r="B44" s="12">
         <v>0.4375</v>
@@ -2334,10 +2334,10 @@
         <v>0.79166666666666663</v>
       </c>
       <c r="D44" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E44" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F44" s="12">
         <v>0.4375</v>
@@ -2364,15 +2364,15 @@
         <v>0.83333333333333337</v>
       </c>
       <c r="N44" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="O44" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="45" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A45" s="6" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B45" s="12">
         <v>0.4375</v>
@@ -2381,10 +2381,10 @@
         <v>0.79166666666666663</v>
       </c>
       <c r="D45" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E45" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F45" s="12">
         <v>0.4375</v>
@@ -2411,15 +2411,15 @@
         <v>0.83333333333333337</v>
       </c>
       <c r="N45" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="O45" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="46" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A46" s="6" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B46" s="12">
         <v>0.4375</v>
@@ -2428,10 +2428,10 @@
         <v>0.79166666666666663</v>
       </c>
       <c r="D46" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E46" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F46" s="12">
         <v>0.4375</v>
@@ -2458,15 +2458,15 @@
         <v>0.83333333333333337</v>
       </c>
       <c r="N46" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="O46" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="47" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A47" s="6" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B47" s="12">
         <v>0.4375</v>
@@ -2475,10 +2475,10 @@
         <v>0.79166666666666663</v>
       </c>
       <c r="D47" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E47" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F47" s="12">
         <v>0.4375</v>
@@ -2505,15 +2505,15 @@
         <v>0.83333333333333337</v>
       </c>
       <c r="N47" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="O47" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="48" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A48" s="6" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B48" s="12">
         <v>0.4375</v>
@@ -2522,10 +2522,10 @@
         <v>0.79166666666666663</v>
       </c>
       <c r="D48" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E48" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F48" s="12">
         <v>0.4375</v>
@@ -2552,15 +2552,15 @@
         <v>0.83333333333333337</v>
       </c>
       <c r="N48" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="O48" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="49" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A49" s="14" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B49" s="12">
         <v>0.4375</v>
@@ -2569,10 +2569,10 @@
         <v>0.79166666666666663</v>
       </c>
       <c r="D49" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E49" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F49" s="12">
         <v>0.4375</v>
@@ -2599,15 +2599,15 @@
         <v>0.83333333333333337</v>
       </c>
       <c r="N49" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="O49" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="52" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B52" s="15" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C52" s="15"/>
       <c r="D52" s="15"/>
@@ -2718,16 +2718,16 @@
         <v>0.79166666666666663</v>
       </c>
       <c r="F55" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="G55" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="H55" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="I55" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="J55" s="12">
         <v>0.41666666666666669</v>
@@ -2765,16 +2765,16 @@
         <v>0.83333333333333337</v>
       </c>
       <c r="F56" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="G56" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="H56" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="I56" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="J56" s="12">
         <v>0.41666666666666669</v>
@@ -2812,16 +2812,16 @@
         <v>0.79166666666666663</v>
       </c>
       <c r="F57" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="G57" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="H57" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="I57" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="J57" s="12">
         <v>0.41666666666666669</v>
@@ -2859,16 +2859,16 @@
         <v>0.83333333333333337</v>
       </c>
       <c r="F58" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="G58" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="H58" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="I58" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="J58" s="12">
         <v>0.41666666666666669</v>
@@ -2906,16 +2906,16 @@
         <v>0.79166666666666663</v>
       </c>
       <c r="F59" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="G59" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="H59" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="I59" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="J59" s="12">
         <v>0.41666666666666669</v>
@@ -2953,16 +2953,16 @@
         <v>0.79166666666666663</v>
       </c>
       <c r="F60" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="G60" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="H60" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="I60" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="J60" s="12">
         <v>0.41666666666666669</v>
@@ -2985,7 +2985,7 @@
     </row>
     <row r="61" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A61" s="6" t="s">
-        <v>9</v>
+        <v>19</v>
       </c>
       <c r="B61" s="12">
         <v>0.4375</v>
@@ -3000,16 +3000,16 @@
         <v>0.79166666666666663</v>
       </c>
       <c r="F61" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="G61" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="H61" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="I61" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="J61" s="12">
         <v>0.41666666666666669</v>
@@ -3032,7 +3032,7 @@
     </row>
     <row r="62" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A62" s="6" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B62" s="12">
         <v>0.4375</v>
@@ -3047,16 +3047,16 @@
         <v>0.79166666666666663</v>
       </c>
       <c r="F62" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="G62" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="H62" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="I62" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="J62" s="12">
         <v>0.41666666666666669</v>
@@ -3079,7 +3079,7 @@
     </row>
     <row r="63" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A63" s="6" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B63" s="12">
         <v>0.4375</v>
@@ -3094,16 +3094,16 @@
         <v>0.79166666666666663</v>
       </c>
       <c r="F63" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="G63" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="H63" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="I63" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="J63" s="12">
         <v>0.41666666666666669</v>
@@ -3126,7 +3126,7 @@
     </row>
     <row r="64" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A64" s="6" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B64" s="12">
         <v>0.4375</v>
@@ -3141,16 +3141,16 @@
         <v>0.79166666666666663</v>
       </c>
       <c r="F64" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="G64" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="H64" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="I64" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="J64" s="12">
         <v>0.41666666666666669</v>
@@ -3173,7 +3173,7 @@
     </row>
     <row r="65" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A65" s="6" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B65" s="12">
         <v>0.4375</v>
@@ -3188,16 +3188,16 @@
         <v>0.79166666666666663</v>
       </c>
       <c r="F65" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="G65" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="H65" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="I65" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="J65" s="12">
         <v>0.41666666666666669</v>
@@ -3220,7 +3220,7 @@
     </row>
     <row r="66" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A66" s="14" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B66" s="12">
         <v>0.4375</v>
@@ -3235,16 +3235,16 @@
         <v>0.79166666666666663</v>
       </c>
       <c r="F66" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="G66" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="H66" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="I66" s="11" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="J66" s="12">
         <v>0.41666666666666669</v>

</xml_diff>

<commit_message>
Actualizar horarios.xlsx (mas informacion)
</commit_message>
<xml_diff>
--- a/horarios.xlsx
+++ b/horarios.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Dreame\Desktop\Claude\Dreame\Turnos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F71C0268-9425-466C-A616-8870E8896F72}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{92B3F74F-28B6-416A-91B8-151C21437A34}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="288" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="299" uniqueCount="22">
   <si>
     <t>Promotor</t>
   </si>
@@ -99,6 +99,9 @@
   </si>
   <si>
     <t>MATIAS BERENGUELA</t>
+  </si>
+  <si>
+    <t>DIEGO MARTINEZ</t>
   </si>
 </sst>
 </file>
@@ -604,7 +607,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3DB7FB46-34C8-4ECD-A089-0D01F6EF7C8B}">
-  <dimension ref="A1:R68"/>
+  <dimension ref="A1:R71"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="34.33203125" bestFit="1" customWidth="1"/>
@@ -1889,441 +1892,433 @@
         <v>10</v>
       </c>
     </row>
-    <row r="32" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A32" s="14" t="s">
+    <row r="32" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A32" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="B32" s="11"/>
+      <c r="C32" s="11"/>
+      <c r="D32" s="12"/>
+      <c r="E32" s="12"/>
+      <c r="F32" s="12">
+        <v>0.4375</v>
+      </c>
+      <c r="G32" s="12">
+        <v>0.79166666666666663</v>
+      </c>
+      <c r="H32" s="12">
+        <v>0.41666666666666669</v>
+      </c>
+      <c r="I32" s="12">
+        <v>0.83333333333333337</v>
+      </c>
+      <c r="J32" s="12">
+        <v>0.41666666666666669</v>
+      </c>
+      <c r="K32" s="12">
+        <v>0.83333333333333337</v>
+      </c>
+      <c r="L32" s="12">
+        <v>0.41666666666666669</v>
+      </c>
+      <c r="M32" s="12">
+        <v>0.83333333333333337</v>
+      </c>
+      <c r="N32" s="11" t="s">
+        <v>10</v>
+      </c>
+      <c r="O32" s="11" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="33" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A33" s="14" t="s">
         <v>11</v>
       </c>
-      <c r="B32" s="11" t="s">
-        <v>10</v>
-      </c>
-      <c r="C32" s="11" t="s">
-        <v>10</v>
-      </c>
-      <c r="D32" s="12">
-        <v>0.4375</v>
-      </c>
-      <c r="E32" s="12">
-        <v>0.79166666666666663</v>
-      </c>
-      <c r="F32" s="12">
-        <v>0.4375</v>
-      </c>
-      <c r="G32" s="12">
-        <v>0.79166666666666663</v>
-      </c>
-      <c r="H32" s="12">
-        <v>0.41666666666666669</v>
-      </c>
-      <c r="I32" s="12">
-        <v>0.83333333333333337</v>
-      </c>
-      <c r="J32" s="12">
-        <v>0.41666666666666669</v>
-      </c>
-      <c r="K32" s="12">
-        <v>0.83333333333333337</v>
-      </c>
-      <c r="L32" s="12">
-        <v>0.41666666666666669</v>
-      </c>
-      <c r="M32" s="12">
-        <v>0.83333333333333337</v>
-      </c>
-      <c r="N32" s="11" t="s">
-        <v>10</v>
-      </c>
-      <c r="O32" s="11" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="35" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B35" s="15" t="s">
+      <c r="B33" s="11" t="s">
+        <v>10</v>
+      </c>
+      <c r="C33" s="11" t="s">
+        <v>10</v>
+      </c>
+      <c r="D33" s="12">
+        <v>0.4375</v>
+      </c>
+      <c r="E33" s="12">
+        <v>0.79166666666666663</v>
+      </c>
+      <c r="F33" s="12">
+        <v>0.4375</v>
+      </c>
+      <c r="G33" s="12">
+        <v>0.79166666666666663</v>
+      </c>
+      <c r="H33" s="12">
+        <v>0.41666666666666669</v>
+      </c>
+      <c r="I33" s="12">
+        <v>0.83333333333333337</v>
+      </c>
+      <c r="J33" s="12">
+        <v>0.41666666666666669</v>
+      </c>
+      <c r="K33" s="12">
+        <v>0.83333333333333337</v>
+      </c>
+      <c r="L33" s="12">
+        <v>0.41666666666666669</v>
+      </c>
+      <c r="M33" s="12">
+        <v>0.83333333333333337</v>
+      </c>
+      <c r="N33" s="11" t="s">
+        <v>10</v>
+      </c>
+      <c r="O33" s="11" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="36" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B36" s="15" t="s">
         <v>8</v>
       </c>
-      <c r="C35" s="15"/>
-      <c r="D35" s="15"/>
-      <c r="E35" s="15"/>
-      <c r="F35" s="15"/>
-      <c r="G35" s="15"/>
-      <c r="H35" s="15"/>
-      <c r="I35" s="15"/>
-      <c r="J35" s="15"/>
-      <c r="K35" s="15"/>
-      <c r="L35" s="15"/>
-      <c r="M35" s="15"/>
-      <c r="N35" s="15"/>
-      <c r="O35" s="15"/>
-    </row>
-    <row r="36" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A36" s="1" t="s">
+      <c r="C36" s="15"/>
+      <c r="D36" s="15"/>
+      <c r="E36" s="15"/>
+      <c r="F36" s="15"/>
+      <c r="G36" s="15"/>
+      <c r="H36" s="15"/>
+      <c r="I36" s="15"/>
+      <c r="J36" s="15"/>
+      <c r="K36" s="15"/>
+      <c r="L36" s="15"/>
+      <c r="M36" s="15"/>
+      <c r="N36" s="15"/>
+      <c r="O36" s="15"/>
+    </row>
+    <row r="37" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A37" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B36" s="16">
+      <c r="B37" s="16">
         <v>46251</v>
       </c>
-      <c r="C36" s="17"/>
-      <c r="D36" s="16">
+      <c r="C37" s="17"/>
+      <c r="D37" s="16">
         <v>46252</v>
       </c>
-      <c r="E36" s="17"/>
-      <c r="F36" s="16">
+      <c r="E37" s="17"/>
+      <c r="F37" s="16">
         <v>46253</v>
       </c>
-      <c r="G36" s="17"/>
-      <c r="H36" s="16">
+      <c r="G37" s="17"/>
+      <c r="H37" s="16">
         <v>46254</v>
       </c>
-      <c r="I36" s="17"/>
-      <c r="J36" s="16">
+      <c r="I37" s="17"/>
+      <c r="J37" s="16">
         <v>46255</v>
       </c>
-      <c r="K36" s="17"/>
-      <c r="L36" s="16">
+      <c r="K37" s="17"/>
+      <c r="L37" s="16">
         <v>46256</v>
       </c>
-      <c r="M36" s="17"/>
-      <c r="N36" s="16">
+      <c r="M37" s="17"/>
+      <c r="N37" s="16">
         <v>46257</v>
       </c>
-      <c r="O36" s="17"/>
-    </row>
-    <row r="37" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A37" s="2"/>
-      <c r="B37" s="7" t="s">
+      <c r="O37" s="17"/>
+    </row>
+    <row r="38" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A38" s="2"/>
+      <c r="B38" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="C37" s="7" t="s">
+      <c r="C38" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="D37" s="8" t="s">
+      <c r="D38" s="8" t="s">
         <v>1</v>
       </c>
-      <c r="E37" s="4" t="s">
+      <c r="E38" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="F37" s="4" t="s">
+      <c r="F38" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="G37" s="4" t="s">
+      <c r="G38" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="H37" s="4" t="s">
+      <c r="H38" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="I37" s="4" t="s">
+      <c r="I38" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="J37" s="4" t="s">
+      <c r="J38" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="K37" s="4" t="s">
+      <c r="K38" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="L37" s="4" t="s">
+      <c r="L38" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="M37" s="4" t="s">
+      <c r="M38" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="N37" s="4" t="s">
+      <c r="N38" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="O37" s="4" t="s">
+      <c r="O38" s="4" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="38" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A38" s="13" t="str">
+    <row r="39" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A39" s="13" t="str">
         <f>+A20</f>
         <v>RAFAEL BUSTOS</v>
       </c>
-      <c r="B38" s="10">
-        <v>0.4375</v>
-      </c>
-      <c r="C38" s="10">
-        <v>0.79166666666666663</v>
-      </c>
-      <c r="D38" s="9" t="s">
-        <v>10</v>
-      </c>
-      <c r="E38" s="11" t="s">
-        <v>10</v>
-      </c>
-      <c r="F38" s="12">
-        <v>0.4375</v>
-      </c>
-      <c r="G38" s="12">
-        <v>0.79166666666666663</v>
-      </c>
-      <c r="H38" s="12">
-        <v>0.41666666666666669</v>
-      </c>
-      <c r="I38" s="12">
-        <v>0.83333333333333337</v>
-      </c>
-      <c r="J38" s="12">
-        <v>0.41666666666666669</v>
-      </c>
-      <c r="K38" s="12">
-        <v>0.83333333333333337</v>
-      </c>
-      <c r="L38" s="12">
-        <v>0.41666666666666669</v>
-      </c>
-      <c r="M38" s="12">
-        <v>0.83333333333333337</v>
-      </c>
-      <c r="N38" s="11" t="s">
-        <v>10</v>
-      </c>
-      <c r="O38" s="11" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="39" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A39" s="6" t="str">
+      <c r="B39" s="10">
+        <v>0.4375</v>
+      </c>
+      <c r="C39" s="10">
+        <v>0.79166666666666663</v>
+      </c>
+      <c r="D39" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="E39" s="11" t="s">
+        <v>10</v>
+      </c>
+      <c r="F39" s="12">
+        <v>0.4375</v>
+      </c>
+      <c r="G39" s="12">
+        <v>0.79166666666666663</v>
+      </c>
+      <c r="H39" s="12">
+        <v>0.41666666666666669</v>
+      </c>
+      <c r="I39" s="12">
+        <v>0.83333333333333337</v>
+      </c>
+      <c r="J39" s="12">
+        <v>0.41666666666666669</v>
+      </c>
+      <c r="K39" s="12">
+        <v>0.83333333333333337</v>
+      </c>
+      <c r="L39" s="12">
+        <v>0.41666666666666669</v>
+      </c>
+      <c r="M39" s="12">
+        <v>0.83333333333333337</v>
+      </c>
+      <c r="N39" s="11" t="s">
+        <v>10</v>
+      </c>
+      <c r="O39" s="11" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="40" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A40" s="6" t="str">
         <f>+A21</f>
         <v xml:space="preserve">GEISSLEN ERICES </v>
       </c>
-      <c r="B39" s="12">
-        <v>0.4375</v>
-      </c>
-      <c r="C39" s="12">
-        <v>0.79166666666666663</v>
-      </c>
-      <c r="D39" s="11" t="s">
-        <v>10</v>
-      </c>
-      <c r="E39" s="11" t="s">
-        <v>10</v>
-      </c>
-      <c r="F39" s="12">
-        <v>0.4375</v>
-      </c>
-      <c r="G39" s="12">
-        <v>0.79166666666666663</v>
-      </c>
-      <c r="H39" s="12">
-        <v>0.41666666666666669</v>
-      </c>
-      <c r="I39" s="12">
-        <v>0.83333333333333337</v>
-      </c>
-      <c r="J39" s="12">
-        <v>0.41666666666666669</v>
-      </c>
-      <c r="K39" s="12">
-        <v>0.83333333333333337</v>
-      </c>
-      <c r="L39" s="12">
-        <v>0.41666666666666669</v>
-      </c>
-      <c r="M39" s="12">
-        <v>0.83333333333333337</v>
-      </c>
-      <c r="N39" s="11" t="s">
-        <v>10</v>
-      </c>
-      <c r="O39" s="11" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="40" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A40" s="6" t="str">
+      <c r="B40" s="12">
+        <v>0.4375</v>
+      </c>
+      <c r="C40" s="12">
+        <v>0.79166666666666663</v>
+      </c>
+      <c r="D40" s="11" t="s">
+        <v>10</v>
+      </c>
+      <c r="E40" s="11" t="s">
+        <v>10</v>
+      </c>
+      <c r="F40" s="12">
+        <v>0.4375</v>
+      </c>
+      <c r="G40" s="12">
+        <v>0.79166666666666663</v>
+      </c>
+      <c r="H40" s="12">
+        <v>0.41666666666666669</v>
+      </c>
+      <c r="I40" s="12">
+        <v>0.83333333333333337</v>
+      </c>
+      <c r="J40" s="12">
+        <v>0.41666666666666669</v>
+      </c>
+      <c r="K40" s="12">
+        <v>0.83333333333333337</v>
+      </c>
+      <c r="L40" s="12">
+        <v>0.41666666666666669</v>
+      </c>
+      <c r="M40" s="12">
+        <v>0.83333333333333337</v>
+      </c>
+      <c r="N40" s="11" t="s">
+        <v>10</v>
+      </c>
+      <c r="O40" s="11" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="41" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A41" s="6" t="str">
         <f>+A22</f>
         <v>MAXIMILIANO MEDINA</v>
       </c>
-      <c r="B40" s="12">
-        <v>0.4375</v>
-      </c>
-      <c r="C40" s="12">
-        <v>0.79166666666666663</v>
-      </c>
-      <c r="D40" s="11" t="s">
-        <v>10</v>
-      </c>
-      <c r="E40" s="11" t="s">
-        <v>10</v>
-      </c>
-      <c r="F40" s="12">
-        <v>0.4375</v>
-      </c>
-      <c r="G40" s="12">
-        <v>0.79166666666666663</v>
-      </c>
-      <c r="H40" s="12">
-        <v>0.41666666666666669</v>
-      </c>
-      <c r="I40" s="12">
-        <v>0.83333333333333337</v>
-      </c>
-      <c r="J40" s="12">
-        <v>0.41666666666666669</v>
-      </c>
-      <c r="K40" s="12">
-        <v>0.83333333333333337</v>
-      </c>
-      <c r="L40" s="12">
-        <v>0.41666666666666669</v>
-      </c>
-      <c r="M40" s="12">
-        <v>0.83333333333333337</v>
-      </c>
-      <c r="N40" s="11" t="s">
-        <v>10</v>
-      </c>
-      <c r="O40" s="11" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="41" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A41" s="6" t="str">
+      <c r="B41" s="12">
+        <v>0.4375</v>
+      </c>
+      <c r="C41" s="12">
+        <v>0.79166666666666663</v>
+      </c>
+      <c r="D41" s="11" t="s">
+        <v>10</v>
+      </c>
+      <c r="E41" s="11" t="s">
+        <v>10</v>
+      </c>
+      <c r="F41" s="12">
+        <v>0.4375</v>
+      </c>
+      <c r="G41" s="12">
+        <v>0.79166666666666663</v>
+      </c>
+      <c r="H41" s="12">
+        <v>0.41666666666666669</v>
+      </c>
+      <c r="I41" s="12">
+        <v>0.83333333333333337</v>
+      </c>
+      <c r="J41" s="12">
+        <v>0.41666666666666669</v>
+      </c>
+      <c r="K41" s="12">
+        <v>0.83333333333333337</v>
+      </c>
+      <c r="L41" s="12">
+        <v>0.41666666666666669</v>
+      </c>
+      <c r="M41" s="12">
+        <v>0.83333333333333337</v>
+      </c>
+      <c r="N41" s="11" t="s">
+        <v>10</v>
+      </c>
+      <c r="O41" s="11" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="42" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A42" s="6" t="str">
         <f>+A23</f>
         <v>LISSETTE MORALES</v>
       </c>
-      <c r="B41" s="12">
-        <v>0.4375</v>
-      </c>
-      <c r="C41" s="12">
-        <v>0.79166666666666663</v>
-      </c>
-      <c r="D41" s="11" t="s">
-        <v>10</v>
-      </c>
-      <c r="E41" s="11" t="s">
-        <v>10</v>
-      </c>
-      <c r="F41" s="12">
-        <v>0.4375</v>
-      </c>
-      <c r="G41" s="12">
-        <v>0.79166666666666663</v>
-      </c>
-      <c r="H41" s="12">
-        <v>0.41666666666666669</v>
-      </c>
-      <c r="I41" s="12">
-        <v>0.83333333333333337</v>
-      </c>
-      <c r="J41" s="12">
-        <v>0.41666666666666669</v>
-      </c>
-      <c r="K41" s="12">
-        <v>0.83333333333333337</v>
-      </c>
-      <c r="L41" s="12">
-        <v>0.41666666666666669</v>
-      </c>
-      <c r="M41" s="12">
-        <v>0.83333333333333337</v>
-      </c>
-      <c r="N41" s="11" t="s">
-        <v>10</v>
-      </c>
-      <c r="O41" s="11" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="42" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A42" s="6" t="str">
+      <c r="B42" s="12">
+        <v>0.4375</v>
+      </c>
+      <c r="C42" s="12">
+        <v>0.79166666666666663</v>
+      </c>
+      <c r="D42" s="11" t="s">
+        <v>10</v>
+      </c>
+      <c r="E42" s="11" t="s">
+        <v>10</v>
+      </c>
+      <c r="F42" s="12">
+        <v>0.4375</v>
+      </c>
+      <c r="G42" s="12">
+        <v>0.79166666666666663</v>
+      </c>
+      <c r="H42" s="12">
+        <v>0.41666666666666669</v>
+      </c>
+      <c r="I42" s="12">
+        <v>0.83333333333333337</v>
+      </c>
+      <c r="J42" s="12">
+        <v>0.41666666666666669</v>
+      </c>
+      <c r="K42" s="12">
+        <v>0.83333333333333337</v>
+      </c>
+      <c r="L42" s="12">
+        <v>0.41666666666666669</v>
+      </c>
+      <c r="M42" s="12">
+        <v>0.83333333333333337</v>
+      </c>
+      <c r="N42" s="11" t="s">
+        <v>10</v>
+      </c>
+      <c r="O42" s="11" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="43" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A43" s="6" t="str">
         <f>+A24</f>
         <v xml:space="preserve">CRISTIAN MORALES </v>
       </c>
-      <c r="B42" s="12">
-        <v>0.4375</v>
-      </c>
-      <c r="C42" s="12">
-        <v>0.79166666666666663</v>
-      </c>
-      <c r="D42" s="11" t="s">
-        <v>10</v>
-      </c>
-      <c r="E42" s="11" t="s">
-        <v>10</v>
-      </c>
-      <c r="F42" s="12">
-        <v>0.4375</v>
-      </c>
-      <c r="G42" s="12">
-        <v>0.79166666666666663</v>
-      </c>
-      <c r="H42" s="12">
-        <v>0.41666666666666669</v>
-      </c>
-      <c r="I42" s="12">
-        <v>0.83333333333333337</v>
-      </c>
-      <c r="J42" s="12">
-        <v>0.41666666666666669</v>
-      </c>
-      <c r="K42" s="12">
-        <v>0.83333333333333337</v>
-      </c>
-      <c r="L42" s="12">
-        <v>0.41666666666666669</v>
-      </c>
-      <c r="M42" s="12">
-        <v>0.83333333333333337</v>
-      </c>
-      <c r="N42" s="11" t="s">
-        <v>10</v>
-      </c>
-      <c r="O42" s="11" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="43" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A43" s="6" t="str">
+      <c r="B43" s="12">
+        <v>0.4375</v>
+      </c>
+      <c r="C43" s="12">
+        <v>0.79166666666666663</v>
+      </c>
+      <c r="D43" s="11" t="s">
+        <v>10</v>
+      </c>
+      <c r="E43" s="11" t="s">
+        <v>10</v>
+      </c>
+      <c r="F43" s="12">
+        <v>0.4375</v>
+      </c>
+      <c r="G43" s="12">
+        <v>0.79166666666666663</v>
+      </c>
+      <c r="H43" s="12">
+        <v>0.41666666666666669</v>
+      </c>
+      <c r="I43" s="12">
+        <v>0.83333333333333337</v>
+      </c>
+      <c r="J43" s="12">
+        <v>0.41666666666666669</v>
+      </c>
+      <c r="K43" s="12">
+        <v>0.83333333333333337</v>
+      </c>
+      <c r="L43" s="12">
+        <v>0.41666666666666669</v>
+      </c>
+      <c r="M43" s="12">
+        <v>0.83333333333333337</v>
+      </c>
+      <c r="N43" s="11" t="s">
+        <v>10</v>
+      </c>
+      <c r="O43" s="11" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="44" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A44" s="6" t="str">
         <f>+A25</f>
         <v>KARIN NAVIA</v>
       </c>
-      <c r="B43" s="12">
-        <v>0.4375</v>
-      </c>
-      <c r="C43" s="12">
-        <v>0.79166666666666663</v>
-      </c>
-      <c r="D43" s="11" t="s">
-        <v>10</v>
-      </c>
-      <c r="E43" s="11" t="s">
-        <v>10</v>
-      </c>
-      <c r="F43" s="12">
-        <v>0.4375</v>
-      </c>
-      <c r="G43" s="12">
-        <v>0.79166666666666663</v>
-      </c>
-      <c r="H43" s="12">
-        <v>0.41666666666666669</v>
-      </c>
-      <c r="I43" s="12">
-        <v>0.83333333333333337</v>
-      </c>
-      <c r="J43" s="12">
-        <v>0.41666666666666669</v>
-      </c>
-      <c r="K43" s="12">
-        <v>0.83333333333333337</v>
-      </c>
-      <c r="L43" s="12">
-        <v>0.41666666666666669</v>
-      </c>
-      <c r="M43" s="12">
-        <v>0.83333333333333337</v>
-      </c>
-      <c r="N43" s="11" t="s">
-        <v>10</v>
-      </c>
-      <c r="O43" s="11" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="44" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A44" s="6" t="s">
-        <v>12</v>
-      </c>
       <c r="B44" s="12">
         <v>0.4375</v>
       </c>
@@ -2369,103 +2364,103 @@
     </row>
     <row r="45" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A45" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="B45" s="12">
+        <v>0.4375</v>
+      </c>
+      <c r="C45" s="12">
+        <v>0.79166666666666663</v>
+      </c>
+      <c r="D45" s="11" t="s">
+        <v>10</v>
+      </c>
+      <c r="E45" s="11" t="s">
+        <v>10</v>
+      </c>
+      <c r="F45" s="12">
+        <v>0.4375</v>
+      </c>
+      <c r="G45" s="12">
+        <v>0.79166666666666663</v>
+      </c>
+      <c r="H45" s="12">
+        <v>0.41666666666666669</v>
+      </c>
+      <c r="I45" s="12">
+        <v>0.83333333333333337</v>
+      </c>
+      <c r="J45" s="12">
+        <v>0.41666666666666669</v>
+      </c>
+      <c r="K45" s="12">
+        <v>0.83333333333333337</v>
+      </c>
+      <c r="L45" s="12">
+        <v>0.41666666666666669</v>
+      </c>
+      <c r="M45" s="12">
+        <v>0.83333333333333337</v>
+      </c>
+      <c r="N45" s="11" t="s">
+        <v>10</v>
+      </c>
+      <c r="O45" s="11" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="46" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A46" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="B45" s="12">
-        <v>0.4375</v>
-      </c>
-      <c r="C45" s="12">
-        <v>0.79166666666666663</v>
-      </c>
-      <c r="D45" s="11" t="s">
-        <v>10</v>
-      </c>
-      <c r="E45" s="11" t="s">
-        <v>10</v>
-      </c>
-      <c r="F45" s="12">
-        <v>0.4375</v>
-      </c>
-      <c r="G45" s="12">
-        <v>0.79166666666666663</v>
-      </c>
-      <c r="H45" s="12">
-        <v>0.41666666666666669</v>
-      </c>
-      <c r="I45" s="12">
-        <v>0.83333333333333337</v>
-      </c>
-      <c r="J45" s="12">
-        <v>0.41666666666666669</v>
-      </c>
-      <c r="K45" s="12">
-        <v>0.83333333333333337</v>
-      </c>
-      <c r="L45" s="12">
-        <v>0.41666666666666669</v>
-      </c>
-      <c r="M45" s="12">
-        <v>0.83333333333333337</v>
-      </c>
-      <c r="N45" s="11" t="s">
-        <v>10</v>
-      </c>
-      <c r="O45" s="11" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="46" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A46" s="6" t="str">
+      <c r="B46" s="12">
+        <v>0.4375</v>
+      </c>
+      <c r="C46" s="12">
+        <v>0.79166666666666663</v>
+      </c>
+      <c r="D46" s="11" t="s">
+        <v>10</v>
+      </c>
+      <c r="E46" s="11" t="s">
+        <v>10</v>
+      </c>
+      <c r="F46" s="12">
+        <v>0.4375</v>
+      </c>
+      <c r="G46" s="12">
+        <v>0.79166666666666663</v>
+      </c>
+      <c r="H46" s="12">
+        <v>0.41666666666666669</v>
+      </c>
+      <c r="I46" s="12">
+        <v>0.83333333333333337</v>
+      </c>
+      <c r="J46" s="12">
+        <v>0.41666666666666669</v>
+      </c>
+      <c r="K46" s="12">
+        <v>0.83333333333333337</v>
+      </c>
+      <c r="L46" s="12">
+        <v>0.41666666666666669</v>
+      </c>
+      <c r="M46" s="12">
+        <v>0.83333333333333337</v>
+      </c>
+      <c r="N46" s="11" t="s">
+        <v>10</v>
+      </c>
+      <c r="O46" s="11" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="47" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A47" s="6" t="str">
         <f>+A28</f>
         <v>JORDAN RIMMELIN</v>
       </c>
-      <c r="B46" s="12">
-        <v>0.4375</v>
-      </c>
-      <c r="C46" s="12">
-        <v>0.79166666666666663</v>
-      </c>
-      <c r="D46" s="11" t="s">
-        <v>10</v>
-      </c>
-      <c r="E46" s="11" t="s">
-        <v>10</v>
-      </c>
-      <c r="F46" s="12">
-        <v>0.4375</v>
-      </c>
-      <c r="G46" s="12">
-        <v>0.79166666666666663</v>
-      </c>
-      <c r="H46" s="12">
-        <v>0.41666666666666669</v>
-      </c>
-      <c r="I46" s="12">
-        <v>0.83333333333333337</v>
-      </c>
-      <c r="J46" s="12">
-        <v>0.41666666666666669</v>
-      </c>
-      <c r="K46" s="12">
-        <v>0.83333333333333337</v>
-      </c>
-      <c r="L46" s="12">
-        <v>0.41666666666666669</v>
-      </c>
-      <c r="M46" s="12">
-        <v>0.83333333333333337</v>
-      </c>
-      <c r="N46" s="11" t="s">
-        <v>10</v>
-      </c>
-      <c r="O46" s="11" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="47" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A47" s="6" t="s">
-        <v>4</v>
-      </c>
       <c r="B47" s="12">
         <v>0.4375</v>
       </c>
@@ -2511,342 +2506,341 @@
     </row>
     <row r="48" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A48" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="B48" s="12">
+        <v>0.4375</v>
+      </c>
+      <c r="C48" s="12">
+        <v>0.79166666666666663</v>
+      </c>
+      <c r="D48" s="11" t="s">
+        <v>10</v>
+      </c>
+      <c r="E48" s="11" t="s">
+        <v>10</v>
+      </c>
+      <c r="F48" s="12">
+        <v>0.4375</v>
+      </c>
+      <c r="G48" s="12">
+        <v>0.79166666666666663</v>
+      </c>
+      <c r="H48" s="12">
+        <v>0.41666666666666669</v>
+      </c>
+      <c r="I48" s="12">
+        <v>0.83333333333333337</v>
+      </c>
+      <c r="J48" s="12">
+        <v>0.41666666666666669</v>
+      </c>
+      <c r="K48" s="12">
+        <v>0.83333333333333337</v>
+      </c>
+      <c r="L48" s="12">
+        <v>0.41666666666666669</v>
+      </c>
+      <c r="M48" s="12">
+        <v>0.83333333333333337</v>
+      </c>
+      <c r="N48" s="11" t="s">
+        <v>10</v>
+      </c>
+      <c r="O48" s="11" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="49" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A49" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="B48" s="12">
-        <v>0.4375</v>
-      </c>
-      <c r="C48" s="12">
-        <v>0.79166666666666663</v>
-      </c>
-      <c r="D48" s="11" t="s">
-        <v>10</v>
-      </c>
-      <c r="E48" s="11" t="s">
-        <v>10</v>
-      </c>
-      <c r="F48" s="12">
-        <v>0.4375</v>
-      </c>
-      <c r="G48" s="12">
-        <v>0.79166666666666663</v>
-      </c>
-      <c r="H48" s="12">
-        <v>0.41666666666666669</v>
-      </c>
-      <c r="I48" s="12">
-        <v>0.83333333333333337</v>
-      </c>
-      <c r="J48" s="12">
-        <v>0.41666666666666669</v>
-      </c>
-      <c r="K48" s="12">
-        <v>0.83333333333333337</v>
-      </c>
-      <c r="L48" s="12">
-        <v>0.41666666666666669</v>
-      </c>
-      <c r="M48" s="12">
-        <v>0.83333333333333337</v>
-      </c>
-      <c r="N48" s="11" t="s">
-        <v>10</v>
-      </c>
-      <c r="O48" s="11" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="49" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A49" s="6" t="str">
+      <c r="B49" s="12">
+        <v>0.4375</v>
+      </c>
+      <c r="C49" s="12">
+        <v>0.79166666666666663</v>
+      </c>
+      <c r="D49" s="11" t="s">
+        <v>10</v>
+      </c>
+      <c r="E49" s="11" t="s">
+        <v>10</v>
+      </c>
+      <c r="F49" s="12">
+        <v>0.4375</v>
+      </c>
+      <c r="G49" s="12">
+        <v>0.79166666666666663</v>
+      </c>
+      <c r="H49" s="12">
+        <v>0.41666666666666669</v>
+      </c>
+      <c r="I49" s="12">
+        <v>0.83333333333333337</v>
+      </c>
+      <c r="J49" s="12">
+        <v>0.41666666666666669</v>
+      </c>
+      <c r="K49" s="12">
+        <v>0.83333333333333337</v>
+      </c>
+      <c r="L49" s="12">
+        <v>0.41666666666666669</v>
+      </c>
+      <c r="M49" s="12">
+        <v>0.83333333333333337</v>
+      </c>
+      <c r="N49" s="11" t="s">
+        <v>10</v>
+      </c>
+      <c r="O49" s="11" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="50" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A50" s="6" t="str">
         <f>+A31</f>
         <v>MATIAS BERENGUELA</v>
       </c>
-      <c r="B49" s="12">
-        <v>0.4375</v>
-      </c>
-      <c r="C49" s="12">
-        <v>0.79166666666666663</v>
-      </c>
-      <c r="D49" s="11" t="s">
-        <v>10</v>
-      </c>
-      <c r="E49" s="11" t="s">
-        <v>10</v>
-      </c>
-      <c r="F49" s="12">
-        <v>0.4375</v>
-      </c>
-      <c r="G49" s="12">
-        <v>0.79166666666666663</v>
-      </c>
-      <c r="H49" s="12">
-        <v>0.41666666666666669</v>
-      </c>
-      <c r="I49" s="12">
-        <v>0.83333333333333337</v>
-      </c>
-      <c r="J49" s="12">
-        <v>0.41666666666666669</v>
-      </c>
-      <c r="K49" s="12">
-        <v>0.83333333333333337</v>
-      </c>
-      <c r="L49" s="12">
-        <v>0.41666666666666669</v>
-      </c>
-      <c r="M49" s="12">
-        <v>0.83333333333333337</v>
-      </c>
-      <c r="N49" s="11" t="s">
-        <v>10</v>
-      </c>
-      <c r="O49" s="11" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="50" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A50" s="14" t="s">
+      <c r="B50" s="12">
+        <v>0.4375</v>
+      </c>
+      <c r="C50" s="12">
+        <v>0.79166666666666663</v>
+      </c>
+      <c r="D50" s="11" t="s">
+        <v>10</v>
+      </c>
+      <c r="E50" s="11" t="s">
+        <v>10</v>
+      </c>
+      <c r="F50" s="12">
+        <v>0.4375</v>
+      </c>
+      <c r="G50" s="12">
+        <v>0.79166666666666663</v>
+      </c>
+      <c r="H50" s="12">
+        <v>0.41666666666666669</v>
+      </c>
+      <c r="I50" s="12">
+        <v>0.83333333333333337</v>
+      </c>
+      <c r="J50" s="12">
+        <v>0.41666666666666669</v>
+      </c>
+      <c r="K50" s="12">
+        <v>0.83333333333333337</v>
+      </c>
+      <c r="L50" s="12">
+        <v>0.41666666666666669</v>
+      </c>
+      <c r="M50" s="12">
+        <v>0.83333333333333337</v>
+      </c>
+      <c r="N50" s="11" t="s">
+        <v>10</v>
+      </c>
+      <c r="O50" s="11" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="51" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A51" s="6" t="str">
+        <f>+A32</f>
+        <v>DIEGO MARTINEZ</v>
+      </c>
+      <c r="B51" s="12">
+        <v>0.4375</v>
+      </c>
+      <c r="C51" s="12">
+        <v>0.79166666666666663</v>
+      </c>
+      <c r="D51" s="11" t="s">
+        <v>10</v>
+      </c>
+      <c r="E51" s="11" t="s">
+        <v>10</v>
+      </c>
+      <c r="F51" s="12">
+        <v>0.4375</v>
+      </c>
+      <c r="G51" s="12">
+        <v>0.79166666666666663</v>
+      </c>
+      <c r="H51" s="12">
+        <v>0.41666666666666669</v>
+      </c>
+      <c r="I51" s="12">
+        <v>0.83333333333333337</v>
+      </c>
+      <c r="J51" s="12">
+        <v>0.41666666666666669</v>
+      </c>
+      <c r="K51" s="12">
+        <v>0.83333333333333337</v>
+      </c>
+      <c r="L51" s="12">
+        <v>0.41666666666666669</v>
+      </c>
+      <c r="M51" s="12">
+        <v>0.83333333333333337</v>
+      </c>
+      <c r="N51" s="11" t="s">
+        <v>10</v>
+      </c>
+      <c r="O51" s="11" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="52" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A52" s="14" t="s">
         <v>11</v>
       </c>
-      <c r="B50" s="12">
-        <v>0.4375</v>
-      </c>
-      <c r="C50" s="12">
-        <v>0.79166666666666663</v>
-      </c>
-      <c r="D50" s="11" t="s">
-        <v>10</v>
-      </c>
-      <c r="E50" s="11" t="s">
-        <v>10</v>
-      </c>
-      <c r="F50" s="12">
-        <v>0.4375</v>
-      </c>
-      <c r="G50" s="12">
-        <v>0.79166666666666663</v>
-      </c>
-      <c r="H50" s="12">
-        <v>0.41666666666666669</v>
-      </c>
-      <c r="I50" s="12">
-        <v>0.83333333333333337</v>
-      </c>
-      <c r="J50" s="12">
-        <v>0.41666666666666669</v>
-      </c>
-      <c r="K50" s="12">
-        <v>0.83333333333333337</v>
-      </c>
-      <c r="L50" s="12">
-        <v>0.41666666666666669</v>
-      </c>
-      <c r="M50" s="12">
-        <v>0.83333333333333337</v>
-      </c>
-      <c r="N50" s="11" t="s">
-        <v>10</v>
-      </c>
-      <c r="O50" s="11" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="53" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B53" s="15" t="s">
+      <c r="B52" s="12">
+        <v>0.4375</v>
+      </c>
+      <c r="C52" s="12">
+        <v>0.79166666666666663</v>
+      </c>
+      <c r="D52" s="11" t="s">
+        <v>10</v>
+      </c>
+      <c r="E52" s="11" t="s">
+        <v>10</v>
+      </c>
+      <c r="F52" s="12">
+        <v>0.4375</v>
+      </c>
+      <c r="G52" s="12">
+        <v>0.79166666666666663</v>
+      </c>
+      <c r="H52" s="12">
+        <v>0.41666666666666669</v>
+      </c>
+      <c r="I52" s="12">
+        <v>0.83333333333333337</v>
+      </c>
+      <c r="J52" s="12">
+        <v>0.41666666666666669</v>
+      </c>
+      <c r="K52" s="12">
+        <v>0.83333333333333337</v>
+      </c>
+      <c r="L52" s="12">
+        <v>0.41666666666666669</v>
+      </c>
+      <c r="M52" s="12">
+        <v>0.83333333333333337</v>
+      </c>
+      <c r="N52" s="11" t="s">
+        <v>10</v>
+      </c>
+      <c r="O52" s="11" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="55" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B55" s="15" t="s">
         <v>9</v>
       </c>
-      <c r="C53" s="15"/>
-      <c r="D53" s="15"/>
-      <c r="E53" s="15"/>
-      <c r="F53" s="15"/>
-      <c r="G53" s="15"/>
-      <c r="H53" s="15"/>
-      <c r="I53" s="15"/>
-      <c r="J53" s="15"/>
-      <c r="K53" s="15"/>
-      <c r="L53" s="15"/>
-      <c r="M53" s="15"/>
-      <c r="N53" s="15"/>
-      <c r="O53" s="15"/>
-    </row>
-    <row r="54" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A54" s="1" t="s">
+      <c r="C55" s="15"/>
+      <c r="D55" s="15"/>
+      <c r="E55" s="15"/>
+      <c r="F55" s="15"/>
+      <c r="G55" s="15"/>
+      <c r="H55" s="15"/>
+      <c r="I55" s="15"/>
+      <c r="J55" s="15"/>
+      <c r="K55" s="15"/>
+      <c r="L55" s="15"/>
+      <c r="M55" s="15"/>
+      <c r="N55" s="15"/>
+      <c r="O55" s="15"/>
+    </row>
+    <row r="56" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A56" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B54" s="16">
+      <c r="B56" s="16">
         <v>46258</v>
       </c>
-      <c r="C54" s="17"/>
-      <c r="D54" s="16">
+      <c r="C56" s="17"/>
+      <c r="D56" s="16">
         <v>46259</v>
       </c>
-      <c r="E54" s="17"/>
-      <c r="F54" s="16">
+      <c r="E56" s="17"/>
+      <c r="F56" s="16">
         <v>46260</v>
       </c>
-      <c r="G54" s="17"/>
-      <c r="H54" s="16">
+      <c r="G56" s="17"/>
+      <c r="H56" s="16">
         <v>46261</v>
       </c>
-      <c r="I54" s="17"/>
-      <c r="J54" s="16">
+      <c r="I56" s="17"/>
+      <c r="J56" s="16">
         <v>46262</v>
       </c>
-      <c r="K54" s="17"/>
-      <c r="L54" s="16">
+      <c r="K56" s="17"/>
+      <c r="L56" s="16">
         <v>46263</v>
       </c>
-      <c r="M54" s="17"/>
-      <c r="N54" s="16">
+      <c r="M56" s="17"/>
+      <c r="N56" s="16">
         <v>46264</v>
       </c>
-      <c r="O54" s="17"/>
-    </row>
-    <row r="55" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A55" s="2"/>
-      <c r="B55" s="7" t="s">
+      <c r="O56" s="17"/>
+    </row>
+    <row r="57" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A57" s="2"/>
+      <c r="B57" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="C55" s="7" t="s">
+      <c r="C57" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="D55" s="8" t="s">
+      <c r="D57" s="8" t="s">
         <v>1</v>
       </c>
-      <c r="E55" s="8" t="s">
+      <c r="E57" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="F55" s="8" t="s">
+      <c r="F57" s="8" t="s">
         <v>1</v>
       </c>
-      <c r="G55" s="8" t="s">
+      <c r="G57" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="H55" s="8" t="s">
+      <c r="H57" s="8" t="s">
         <v>1</v>
       </c>
-      <c r="I55" s="8" t="s">
+      <c r="I57" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="J55" s="8" t="s">
+      <c r="J57" s="8" t="s">
         <v>1</v>
       </c>
-      <c r="K55" s="8" t="s">
+      <c r="K57" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="L55" s="8" t="s">
+      <c r="L57" s="8" t="s">
         <v>1</v>
       </c>
-      <c r="M55" s="8" t="s">
+      <c r="M57" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="N55" s="8" t="s">
+      <c r="N57" s="8" t="s">
         <v>1</v>
       </c>
-      <c r="O55" s="8" t="s">
+      <c r="O57" s="8" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="56" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A56" s="13" t="str">
-        <f>+A38</f>
+    <row r="58" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A58" s="13" t="str">
+        <f t="shared" ref="A58:A63" si="0">+A39</f>
         <v>RAFAEL BUSTOS</v>
-      </c>
-      <c r="B56" s="12">
-        <v>0.4375</v>
-      </c>
-      <c r="C56" s="12">
-        <v>0.79166666666666663</v>
-      </c>
-      <c r="D56" s="12">
-        <v>0.4375</v>
-      </c>
-      <c r="E56" s="12">
-        <v>0.79166666666666663</v>
-      </c>
-      <c r="F56" s="11" t="s">
-        <v>10</v>
-      </c>
-      <c r="G56" s="11" t="s">
-        <v>10</v>
-      </c>
-      <c r="H56" s="11" t="s">
-        <v>10</v>
-      </c>
-      <c r="I56" s="11" t="s">
-        <v>10</v>
-      </c>
-      <c r="J56" s="12">
-        <v>0.41666666666666669</v>
-      </c>
-      <c r="K56" s="12">
-        <v>0.83333333333333337</v>
-      </c>
-      <c r="L56" s="12">
-        <v>0.41666666666666669</v>
-      </c>
-      <c r="M56" s="12">
-        <v>0.83333333333333337</v>
-      </c>
-      <c r="N56" s="12">
-        <v>0.41666666666666669</v>
-      </c>
-      <c r="O56" s="12">
-        <v>0.83333333333333337</v>
-      </c>
-    </row>
-    <row r="57" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A57" s="6" t="str">
-        <f>+A39</f>
-        <v xml:space="preserve">GEISSLEN ERICES </v>
-      </c>
-      <c r="B57" s="12">
-        <v>0.4375</v>
-      </c>
-      <c r="C57" s="12">
-        <v>0.79166666666666663</v>
-      </c>
-      <c r="D57" s="12">
-        <v>0.41666666666666669</v>
-      </c>
-      <c r="E57" s="12">
-        <v>0.83333333333333337</v>
-      </c>
-      <c r="F57" s="11" t="s">
-        <v>10</v>
-      </c>
-      <c r="G57" s="11" t="s">
-        <v>10</v>
-      </c>
-      <c r="H57" s="11" t="s">
-        <v>10</v>
-      </c>
-      <c r="I57" s="11" t="s">
-        <v>10</v>
-      </c>
-      <c r="J57" s="12">
-        <v>0.41666666666666669</v>
-      </c>
-      <c r="K57" s="12">
-        <v>0.83333333333333337</v>
-      </c>
-      <c r="L57" s="12">
-        <v>0.41666666666666669</v>
-      </c>
-      <c r="M57" s="12">
-        <v>0.83333333333333337</v>
-      </c>
-      <c r="N57" s="12">
-        <v>0.41666666666666669</v>
-      </c>
-      <c r="O57" s="12">
-        <v>0.77083333333333337</v>
-      </c>
-    </row>
-    <row r="58" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A58" s="6" t="str">
-        <f>+A40</f>
-        <v>MAXIMILIANO MEDINA</v>
       </c>
       <c r="B58" s="12">
         <v>0.4375</v>
@@ -2893,8 +2887,8 @@
     </row>
     <row r="59" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A59" s="6" t="str">
-        <f>+A41</f>
-        <v>LISSETTE MORALES</v>
+        <f t="shared" si="0"/>
+        <v xml:space="preserve">GEISSLEN ERICES </v>
       </c>
       <c r="B59" s="12">
         <v>0.4375</v>
@@ -2941,8 +2935,8 @@
     </row>
     <row r="60" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A60" s="6" t="str">
-        <f>+A42</f>
-        <v xml:space="preserve">CRISTIAN MORALES </v>
+        <f t="shared" si="0"/>
+        <v>MAXIMILIANO MEDINA</v>
       </c>
       <c r="B60" s="12">
         <v>0.4375</v>
@@ -2989,150 +2983,151 @@
     </row>
     <row r="61" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A61" s="6" t="str">
-        <f>+A43</f>
+        <f t="shared" si="0"/>
+        <v>LISSETTE MORALES</v>
+      </c>
+      <c r="B61" s="12">
+        <v>0.4375</v>
+      </c>
+      <c r="C61" s="12">
+        <v>0.79166666666666663</v>
+      </c>
+      <c r="D61" s="12">
+        <v>0.41666666666666669</v>
+      </c>
+      <c r="E61" s="12">
+        <v>0.83333333333333337</v>
+      </c>
+      <c r="F61" s="11" t="s">
+        <v>10</v>
+      </c>
+      <c r="G61" s="11" t="s">
+        <v>10</v>
+      </c>
+      <c r="H61" s="11" t="s">
+        <v>10</v>
+      </c>
+      <c r="I61" s="11" t="s">
+        <v>10</v>
+      </c>
+      <c r="J61" s="12">
+        <v>0.41666666666666669</v>
+      </c>
+      <c r="K61" s="12">
+        <v>0.83333333333333337</v>
+      </c>
+      <c r="L61" s="12">
+        <v>0.41666666666666669</v>
+      </c>
+      <c r="M61" s="12">
+        <v>0.83333333333333337</v>
+      </c>
+      <c r="N61" s="12">
+        <v>0.41666666666666669</v>
+      </c>
+      <c r="O61" s="12">
+        <v>0.77083333333333337</v>
+      </c>
+    </row>
+    <row r="62" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A62" s="6" t="str">
+        <f t="shared" si="0"/>
+        <v xml:space="preserve">CRISTIAN MORALES </v>
+      </c>
+      <c r="B62" s="12">
+        <v>0.4375</v>
+      </c>
+      <c r="C62" s="12">
+        <v>0.79166666666666663</v>
+      </c>
+      <c r="D62" s="12">
+        <v>0.4375</v>
+      </c>
+      <c r="E62" s="12">
+        <v>0.79166666666666663</v>
+      </c>
+      <c r="F62" s="11" t="s">
+        <v>10</v>
+      </c>
+      <c r="G62" s="11" t="s">
+        <v>10</v>
+      </c>
+      <c r="H62" s="11" t="s">
+        <v>10</v>
+      </c>
+      <c r="I62" s="11" t="s">
+        <v>10</v>
+      </c>
+      <c r="J62" s="12">
+        <v>0.41666666666666669</v>
+      </c>
+      <c r="K62" s="12">
+        <v>0.83333333333333337</v>
+      </c>
+      <c r="L62" s="12">
+        <v>0.41666666666666669</v>
+      </c>
+      <c r="M62" s="12">
+        <v>0.83333333333333337</v>
+      </c>
+      <c r="N62" s="12">
+        <v>0.41666666666666669</v>
+      </c>
+      <c r="O62" s="12">
+        <v>0.83333333333333337</v>
+      </c>
+    </row>
+    <row r="63" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A63" s="6" t="str">
+        <f t="shared" si="0"/>
         <v>KARIN NAVIA</v>
       </c>
-      <c r="B61" s="12">
-        <v>0.4375</v>
-      </c>
-      <c r="C61" s="12">
-        <v>0.79166666666666663</v>
-      </c>
-      <c r="D61" s="12">
-        <v>0.4375</v>
-      </c>
-      <c r="E61" s="12">
-        <v>0.79166666666666663</v>
-      </c>
-      <c r="F61" s="11" t="s">
-        <v>10</v>
-      </c>
-      <c r="G61" s="11" t="s">
-        <v>10</v>
-      </c>
-      <c r="H61" s="11" t="s">
-        <v>10</v>
-      </c>
-      <c r="I61" s="11" t="s">
-        <v>10</v>
-      </c>
-      <c r="J61" s="12">
-        <v>0.41666666666666669</v>
-      </c>
-      <c r="K61" s="12">
-        <v>0.83333333333333337</v>
-      </c>
-      <c r="L61" s="12">
-        <v>0.41666666666666669</v>
-      </c>
-      <c r="M61" s="12">
-        <v>0.83333333333333337</v>
-      </c>
-      <c r="N61" s="12">
-        <v>0.41666666666666669</v>
-      </c>
-      <c r="O61" s="12">
-        <v>0.83333333333333337</v>
-      </c>
-    </row>
-    <row r="62" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A62" s="6" t="s">
+      <c r="B63" s="12">
+        <v>0.4375</v>
+      </c>
+      <c r="C63" s="12">
+        <v>0.79166666666666663</v>
+      </c>
+      <c r="D63" s="12">
+        <v>0.4375</v>
+      </c>
+      <c r="E63" s="12">
+        <v>0.79166666666666663</v>
+      </c>
+      <c r="F63" s="11" t="s">
+        <v>10</v>
+      </c>
+      <c r="G63" s="11" t="s">
+        <v>10</v>
+      </c>
+      <c r="H63" s="11" t="s">
+        <v>10</v>
+      </c>
+      <c r="I63" s="11" t="s">
+        <v>10</v>
+      </c>
+      <c r="J63" s="12">
+        <v>0.41666666666666669</v>
+      </c>
+      <c r="K63" s="12">
+        <v>0.83333333333333337</v>
+      </c>
+      <c r="L63" s="12">
+        <v>0.41666666666666669</v>
+      </c>
+      <c r="M63" s="12">
+        <v>0.83333333333333337</v>
+      </c>
+      <c r="N63" s="12">
+        <v>0.41666666666666669</v>
+      </c>
+      <c r="O63" s="12">
+        <v>0.83333333333333337</v>
+      </c>
+    </row>
+    <row r="64" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A64" s="6" t="s">
         <v>12</v>
-      </c>
-      <c r="B62" s="12">
-        <v>0.4375</v>
-      </c>
-      <c r="C62" s="12">
-        <v>0.79166666666666663</v>
-      </c>
-      <c r="D62" s="12">
-        <v>0.4375</v>
-      </c>
-      <c r="E62" s="12">
-        <v>0.79166666666666663</v>
-      </c>
-      <c r="F62" s="11" t="s">
-        <v>10</v>
-      </c>
-      <c r="G62" s="11" t="s">
-        <v>10</v>
-      </c>
-      <c r="H62" s="11" t="s">
-        <v>10</v>
-      </c>
-      <c r="I62" s="11" t="s">
-        <v>10</v>
-      </c>
-      <c r="J62" s="12">
-        <v>0.41666666666666669</v>
-      </c>
-      <c r="K62" s="12">
-        <v>0.83333333333333337</v>
-      </c>
-      <c r="L62" s="12">
-        <v>0.41666666666666669</v>
-      </c>
-      <c r="M62" s="12">
-        <v>0.83333333333333337</v>
-      </c>
-      <c r="N62" s="12">
-        <v>0.41666666666666669</v>
-      </c>
-      <c r="O62" s="12">
-        <v>0.83333333333333337</v>
-      </c>
-    </row>
-    <row r="63" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A63" s="6" t="s">
-        <v>3</v>
-      </c>
-      <c r="B63" s="12">
-        <v>0.4375</v>
-      </c>
-      <c r="C63" s="12">
-        <v>0.79166666666666663</v>
-      </c>
-      <c r="D63" s="12">
-        <v>0.4375</v>
-      </c>
-      <c r="E63" s="12">
-        <v>0.79166666666666663</v>
-      </c>
-      <c r="F63" s="11" t="s">
-        <v>10</v>
-      </c>
-      <c r="G63" s="11" t="s">
-        <v>10</v>
-      </c>
-      <c r="H63" s="11" t="s">
-        <v>10</v>
-      </c>
-      <c r="I63" s="11" t="s">
-        <v>10</v>
-      </c>
-      <c r="J63" s="12">
-        <v>0.41666666666666669</v>
-      </c>
-      <c r="K63" s="12">
-        <v>0.83333333333333337</v>
-      </c>
-      <c r="L63" s="12">
-        <v>0.41666666666666669</v>
-      </c>
-      <c r="M63" s="12">
-        <v>0.83333333333333337</v>
-      </c>
-      <c r="N63" s="12">
-        <v>0.41666666666666669</v>
-      </c>
-      <c r="O63" s="12">
-        <v>0.83333333333333337</v>
-      </c>
-    </row>
-    <row r="64" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A64" s="6" t="str">
-        <f>+A46</f>
-        <v>JORDAN RIMMELIN</v>
       </c>
       <c r="B64" s="12">
         <v>0.4375</v>
@@ -3179,211 +3174,346 @@
     </row>
     <row r="65" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A65" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="B65" s="12">
+        <v>0.4375</v>
+      </c>
+      <c r="C65" s="12">
+        <v>0.79166666666666663</v>
+      </c>
+      <c r="D65" s="12">
+        <v>0.4375</v>
+      </c>
+      <c r="E65" s="12">
+        <v>0.79166666666666663</v>
+      </c>
+      <c r="F65" s="11" t="s">
+        <v>10</v>
+      </c>
+      <c r="G65" s="11" t="s">
+        <v>10</v>
+      </c>
+      <c r="H65" s="11" t="s">
+        <v>10</v>
+      </c>
+      <c r="I65" s="11" t="s">
+        <v>10</v>
+      </c>
+      <c r="J65" s="12">
+        <v>0.41666666666666669</v>
+      </c>
+      <c r="K65" s="12">
+        <v>0.83333333333333337</v>
+      </c>
+      <c r="L65" s="12">
+        <v>0.41666666666666669</v>
+      </c>
+      <c r="M65" s="12">
+        <v>0.83333333333333337</v>
+      </c>
+      <c r="N65" s="12">
+        <v>0.41666666666666669</v>
+      </c>
+      <c r="O65" s="12">
+        <v>0.83333333333333337</v>
+      </c>
+    </row>
+    <row r="66" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A66" s="6" t="str">
+        <f>+A47</f>
+        <v>JORDAN RIMMELIN</v>
+      </c>
+      <c r="B66" s="12">
+        <v>0.4375</v>
+      </c>
+      <c r="C66" s="12">
+        <v>0.79166666666666663</v>
+      </c>
+      <c r="D66" s="12">
+        <v>0.4375</v>
+      </c>
+      <c r="E66" s="12">
+        <v>0.79166666666666663</v>
+      </c>
+      <c r="F66" s="11" t="s">
+        <v>10</v>
+      </c>
+      <c r="G66" s="11" t="s">
+        <v>10</v>
+      </c>
+      <c r="H66" s="11" t="s">
+        <v>10</v>
+      </c>
+      <c r="I66" s="11" t="s">
+        <v>10</v>
+      </c>
+      <c r="J66" s="12">
+        <v>0.41666666666666669</v>
+      </c>
+      <c r="K66" s="12">
+        <v>0.83333333333333337</v>
+      </c>
+      <c r="L66" s="12">
+        <v>0.41666666666666669</v>
+      </c>
+      <c r="M66" s="12">
+        <v>0.83333333333333337</v>
+      </c>
+      <c r="N66" s="12">
+        <v>0.41666666666666669</v>
+      </c>
+      <c r="O66" s="12">
+        <v>0.83333333333333337</v>
+      </c>
+    </row>
+    <row r="67" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A67" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="B65" s="12">
-        <v>0.4375</v>
-      </c>
-      <c r="C65" s="12">
-        <v>0.79166666666666663</v>
-      </c>
-      <c r="D65" s="12">
-        <v>0.4375</v>
-      </c>
-      <c r="E65" s="12">
-        <v>0.79166666666666663</v>
-      </c>
-      <c r="F65" s="11" t="s">
-        <v>10</v>
-      </c>
-      <c r="G65" s="11" t="s">
-        <v>10</v>
-      </c>
-      <c r="H65" s="11" t="s">
-        <v>10</v>
-      </c>
-      <c r="I65" s="11" t="s">
-        <v>10</v>
-      </c>
-      <c r="J65" s="12">
-        <v>0.41666666666666669</v>
-      </c>
-      <c r="K65" s="12">
-        <v>0.83333333333333337</v>
-      </c>
-      <c r="L65" s="12">
-        <v>0.41666666666666669</v>
-      </c>
-      <c r="M65" s="12">
-        <v>0.83333333333333337</v>
-      </c>
-      <c r="N65" s="12">
-        <v>0.41666666666666669</v>
-      </c>
-      <c r="O65" s="12">
-        <v>0.83333333333333337</v>
-      </c>
-    </row>
-    <row r="66" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A66" s="6" t="s">
+      <c r="B67" s="12">
+        <v>0.4375</v>
+      </c>
+      <c r="C67" s="12">
+        <v>0.79166666666666663</v>
+      </c>
+      <c r="D67" s="12">
+        <v>0.4375</v>
+      </c>
+      <c r="E67" s="12">
+        <v>0.79166666666666663</v>
+      </c>
+      <c r="F67" s="11" t="s">
+        <v>10</v>
+      </c>
+      <c r="G67" s="11" t="s">
+        <v>10</v>
+      </c>
+      <c r="H67" s="11" t="s">
+        <v>10</v>
+      </c>
+      <c r="I67" s="11" t="s">
+        <v>10</v>
+      </c>
+      <c r="J67" s="12">
+        <v>0.41666666666666669</v>
+      </c>
+      <c r="K67" s="12">
+        <v>0.83333333333333337</v>
+      </c>
+      <c r="L67" s="12">
+        <v>0.41666666666666669</v>
+      </c>
+      <c r="M67" s="12">
+        <v>0.83333333333333337</v>
+      </c>
+      <c r="N67" s="12">
+        <v>0.41666666666666669</v>
+      </c>
+      <c r="O67" s="12">
+        <v>0.83333333333333337</v>
+      </c>
+    </row>
+    <row r="68" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A68" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="B66" s="12">
-        <v>0.4375</v>
-      </c>
-      <c r="C66" s="12">
-        <v>0.79166666666666663</v>
-      </c>
-      <c r="D66" s="12">
-        <v>0.4375</v>
-      </c>
-      <c r="E66" s="12">
-        <v>0.79166666666666663</v>
-      </c>
-      <c r="F66" s="11" t="s">
-        <v>10</v>
-      </c>
-      <c r="G66" s="11" t="s">
-        <v>10</v>
-      </c>
-      <c r="H66" s="11" t="s">
-        <v>10</v>
-      </c>
-      <c r="I66" s="11" t="s">
-        <v>10</v>
-      </c>
-      <c r="J66" s="12">
-        <v>0.41666666666666669</v>
-      </c>
-      <c r="K66" s="12">
-        <v>0.83333333333333337</v>
-      </c>
-      <c r="L66" s="12">
-        <v>0.41666666666666669</v>
-      </c>
-      <c r="M66" s="12">
-        <v>0.83333333333333337</v>
-      </c>
-      <c r="N66" s="12">
-        <v>0.41666666666666669</v>
-      </c>
-      <c r="O66" s="12">
-        <v>0.83333333333333337</v>
-      </c>
-    </row>
-    <row r="67" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A67" s="6" t="str">
-        <f>+A49</f>
+      <c r="B68" s="12">
+        <v>0.4375</v>
+      </c>
+      <c r="C68" s="12">
+        <v>0.79166666666666663</v>
+      </c>
+      <c r="D68" s="12">
+        <v>0.4375</v>
+      </c>
+      <c r="E68" s="12">
+        <v>0.79166666666666663</v>
+      </c>
+      <c r="F68" s="11" t="s">
+        <v>10</v>
+      </c>
+      <c r="G68" s="11" t="s">
+        <v>10</v>
+      </c>
+      <c r="H68" s="11" t="s">
+        <v>10</v>
+      </c>
+      <c r="I68" s="11" t="s">
+        <v>10</v>
+      </c>
+      <c r="J68" s="12">
+        <v>0.41666666666666669</v>
+      </c>
+      <c r="K68" s="12">
+        <v>0.83333333333333337</v>
+      </c>
+      <c r="L68" s="12">
+        <v>0.41666666666666669</v>
+      </c>
+      <c r="M68" s="12">
+        <v>0.83333333333333337</v>
+      </c>
+      <c r="N68" s="12">
+        <v>0.41666666666666669</v>
+      </c>
+      <c r="O68" s="12">
+        <v>0.83333333333333337</v>
+      </c>
+    </row>
+    <row r="69" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A69" s="6" t="str">
+        <f>+A50</f>
         <v>MATIAS BERENGUELA</v>
       </c>
-      <c r="B67" s="12">
-        <v>0.4375</v>
-      </c>
-      <c r="C67" s="12">
-        <v>0.79166666666666663</v>
-      </c>
-      <c r="D67" s="12">
-        <v>0.4375</v>
-      </c>
-      <c r="E67" s="12">
-        <v>0.79166666666666663</v>
-      </c>
-      <c r="F67" s="11" t="s">
-        <v>10</v>
-      </c>
-      <c r="G67" s="11" t="s">
-        <v>10</v>
-      </c>
-      <c r="H67" s="11" t="s">
-        <v>10</v>
-      </c>
-      <c r="I67" s="11" t="s">
-        <v>10</v>
-      </c>
-      <c r="J67" s="12">
-        <v>0.41666666666666669</v>
-      </c>
-      <c r="K67" s="12">
-        <v>0.83333333333333337</v>
-      </c>
-      <c r="L67" s="12">
-        <v>0.41666666666666669</v>
-      </c>
-      <c r="M67" s="12">
-        <v>0.83333333333333337</v>
-      </c>
-      <c r="N67" s="12">
-        <v>0.41666666666666669</v>
-      </c>
-      <c r="O67" s="12">
-        <v>0.83333333333333337</v>
-      </c>
-    </row>
-    <row r="68" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A68" s="14" t="s">
+      <c r="B69" s="12">
+        <v>0.4375</v>
+      </c>
+      <c r="C69" s="12">
+        <v>0.79166666666666663</v>
+      </c>
+      <c r="D69" s="12">
+        <v>0.4375</v>
+      </c>
+      <c r="E69" s="12">
+        <v>0.79166666666666663</v>
+      </c>
+      <c r="F69" s="11" t="s">
+        <v>10</v>
+      </c>
+      <c r="G69" s="11" t="s">
+        <v>10</v>
+      </c>
+      <c r="H69" s="11" t="s">
+        <v>10</v>
+      </c>
+      <c r="I69" s="11" t="s">
+        <v>10</v>
+      </c>
+      <c r="J69" s="12">
+        <v>0.41666666666666669</v>
+      </c>
+      <c r="K69" s="12">
+        <v>0.83333333333333337</v>
+      </c>
+      <c r="L69" s="12">
+        <v>0.41666666666666669</v>
+      </c>
+      <c r="M69" s="12">
+        <v>0.83333333333333337</v>
+      </c>
+      <c r="N69" s="12">
+        <v>0.41666666666666669</v>
+      </c>
+      <c r="O69" s="12">
+        <v>0.83333333333333337</v>
+      </c>
+    </row>
+    <row r="70" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A70" s="6" t="str">
+        <f>+A51</f>
+        <v>DIEGO MARTINEZ</v>
+      </c>
+      <c r="B70" s="12">
+        <v>0.4375</v>
+      </c>
+      <c r="C70" s="12">
+        <v>0.79166666666666663</v>
+      </c>
+      <c r="D70" s="12">
+        <v>0.4375</v>
+      </c>
+      <c r="E70" s="12">
+        <v>0.79166666666666663</v>
+      </c>
+      <c r="F70" s="11" t="s">
+        <v>10</v>
+      </c>
+      <c r="G70" s="11" t="s">
+        <v>10</v>
+      </c>
+      <c r="H70" s="11" t="s">
+        <v>10</v>
+      </c>
+      <c r="I70" s="11" t="s">
+        <v>10</v>
+      </c>
+      <c r="J70" s="12">
+        <v>0.41666666666666669</v>
+      </c>
+      <c r="K70" s="12">
+        <v>0.83333333333333337</v>
+      </c>
+      <c r="L70" s="12">
+        <v>0.41666666666666669</v>
+      </c>
+      <c r="M70" s="12">
+        <v>0.83333333333333337</v>
+      </c>
+      <c r="N70" s="12">
+        <v>0.41666666666666669</v>
+      </c>
+      <c r="O70" s="12">
+        <v>0.83333333333333337</v>
+      </c>
+    </row>
+    <row r="71" spans="1:15" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A71" s="14" t="s">
         <v>11</v>
       </c>
-      <c r="B68" s="12">
-        <v>0.4375</v>
-      </c>
-      <c r="C68" s="12">
-        <v>0.79166666666666663</v>
-      </c>
-      <c r="D68" s="12">
-        <v>0.4375</v>
-      </c>
-      <c r="E68" s="12">
-        <v>0.79166666666666663</v>
-      </c>
-      <c r="F68" s="11" t="s">
-        <v>10</v>
-      </c>
-      <c r="G68" s="11" t="s">
-        <v>10</v>
-      </c>
-      <c r="H68" s="11" t="s">
-        <v>10</v>
-      </c>
-      <c r="I68" s="11" t="s">
-        <v>10</v>
-      </c>
-      <c r="J68" s="12">
-        <v>0.41666666666666669</v>
-      </c>
-      <c r="K68" s="12">
-        <v>0.83333333333333337</v>
-      </c>
-      <c r="L68" s="12">
-        <v>0.41666666666666669</v>
-      </c>
-      <c r="M68" s="12">
-        <v>0.83333333333333337</v>
-      </c>
-      <c r="N68" s="12">
-        <v>0.41666666666666669</v>
-      </c>
-      <c r="O68" s="12">
+      <c r="B71" s="12">
+        <v>0.4375</v>
+      </c>
+      <c r="C71" s="12">
+        <v>0.79166666666666663</v>
+      </c>
+      <c r="D71" s="12">
+        <v>0.4375</v>
+      </c>
+      <c r="E71" s="12">
+        <v>0.79166666666666663</v>
+      </c>
+      <c r="F71" s="11" t="s">
+        <v>10</v>
+      </c>
+      <c r="G71" s="11" t="s">
+        <v>10</v>
+      </c>
+      <c r="H71" s="11" t="s">
+        <v>10</v>
+      </c>
+      <c r="I71" s="11" t="s">
+        <v>10</v>
+      </c>
+      <c r="J71" s="12">
+        <v>0.41666666666666669</v>
+      </c>
+      <c r="K71" s="12">
+        <v>0.83333333333333337</v>
+      </c>
+      <c r="L71" s="12">
+        <v>0.41666666666666669</v>
+      </c>
+      <c r="M71" s="12">
+        <v>0.83333333333333337</v>
+      </c>
+      <c r="N71" s="12">
+        <v>0.41666666666666669</v>
+      </c>
+      <c r="O71" s="12">
         <v>0.83333333333333337</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="32">
-    <mergeCell ref="B53:O53"/>
-    <mergeCell ref="B54:C54"/>
-    <mergeCell ref="D54:E54"/>
-    <mergeCell ref="F54:G54"/>
-    <mergeCell ref="H54:I54"/>
-    <mergeCell ref="J54:K54"/>
-    <mergeCell ref="L54:M54"/>
-    <mergeCell ref="N54:O54"/>
-    <mergeCell ref="B35:O35"/>
-    <mergeCell ref="B36:C36"/>
-    <mergeCell ref="D36:E36"/>
-    <mergeCell ref="F36:G36"/>
-    <mergeCell ref="H36:I36"/>
-    <mergeCell ref="J36:K36"/>
-    <mergeCell ref="L36:M36"/>
-    <mergeCell ref="N36:O36"/>
+    <mergeCell ref="B1:O1"/>
+    <mergeCell ref="B2:C2"/>
+    <mergeCell ref="D2:E2"/>
+    <mergeCell ref="F2:G2"/>
+    <mergeCell ref="H2:I2"/>
+    <mergeCell ref="J2:K2"/>
+    <mergeCell ref="L2:M2"/>
+    <mergeCell ref="N2:O2"/>
     <mergeCell ref="B17:O17"/>
     <mergeCell ref="B18:C18"/>
     <mergeCell ref="D18:E18"/>
@@ -3392,14 +3522,22 @@
     <mergeCell ref="J18:K18"/>
     <mergeCell ref="L18:M18"/>
     <mergeCell ref="N18:O18"/>
-    <mergeCell ref="B1:O1"/>
-    <mergeCell ref="B2:C2"/>
-    <mergeCell ref="D2:E2"/>
-    <mergeCell ref="F2:G2"/>
-    <mergeCell ref="H2:I2"/>
-    <mergeCell ref="J2:K2"/>
-    <mergeCell ref="L2:M2"/>
-    <mergeCell ref="N2:O2"/>
+    <mergeCell ref="B36:O36"/>
+    <mergeCell ref="B37:C37"/>
+    <mergeCell ref="D37:E37"/>
+    <mergeCell ref="F37:G37"/>
+    <mergeCell ref="H37:I37"/>
+    <mergeCell ref="J37:K37"/>
+    <mergeCell ref="L37:M37"/>
+    <mergeCell ref="N37:O37"/>
+    <mergeCell ref="B55:O55"/>
+    <mergeCell ref="B56:C56"/>
+    <mergeCell ref="D56:E56"/>
+    <mergeCell ref="F56:G56"/>
+    <mergeCell ref="H56:I56"/>
+    <mergeCell ref="J56:K56"/>
+    <mergeCell ref="L56:M56"/>
+    <mergeCell ref="N56:O56"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>